<commit_message>
add minor document changes
</commit_message>
<xml_diff>
--- a/data/datasets/graubuenden/GR_22_pressedaten.xlsx
+++ b/data/datasets/graubuenden/GR_22_pressedaten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\semester_6\BA\BA_Thesis\BA_Thesis\data\datasets\graubuenden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_55FE8B61C5CF12547A8C22AC69A1C7800049FF59" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7B7897-F7BF-4CD3-882B-D226DD899343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3220,7 +3220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3251,13 +3251,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3712,7 +3713,7 @@
       <c r="B4" s="3" t="s">
         <v>1019</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -3745,10 +3746,10 @@
       <c r="M4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="N4" s="18" t="s">
+      <c r="N4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="O4" s="19" t="s">
+      <c r="O4" s="18" t="s">
         <v>8</v>
       </c>
     </row>
@@ -11396,7 +11397,7 @@
       <c r="B224" s="3" t="s">
         <v>1019</v>
       </c>
-      <c r="C224" s="18" t="s">
+      <c r="C224" s="19" t="s">
         <v>1</v>
       </c>
       <c r="D224" s="3" t="s">
@@ -11429,10 +11430,10 @@
       <c r="M224" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="N224" s="18" t="s">
+      <c r="N224" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="O224" s="19" t="s">
+      <c r="O224" s="18" t="s">
         <v>8</v>
       </c>
     </row>
@@ -13306,7 +13307,7 @@
       <c r="A3" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="21" t="s">
         <v>157</v>
       </c>
       <c r="C3" s="20" t="s">
@@ -27592,15 +27593,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101007B6A8655AD9ED245B63BD91A39E4310B" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="1bab48deccfafccbcaed9e27982c9d0c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9db63bcbd7c0db8a85e56b2993c8dbc3" ns1:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -27739,6 +27731,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E69716-FCA5-4A3F-BE8C-893EF20583C3}">
   <ds:schemaRefs>
@@ -27750,14 +27751,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6DFDE3A-3299-47BF-89DC-5970B14F6D85}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A42A1E36-70F1-4A21-9F01-F50730240764}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27773,4 +27766,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6DFDE3A-3299-47BF-89DC-5970B14F6D85}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>